<commit_message>
cumulative reserve mu script calculation and output files added
</commit_message>
<xml_diff>
--- a/output/changelog.xlsx
+++ b/output/changelog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imperiallondon-my.sharepoint.com/personal/pgallego_ic_ac_uk/Documents/PhD/Repositories/energy_reserve/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3687" documentId="13_ncr:1_{27CD5DFD-1054-4A33-AFFE-F35EA43968A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{849FC2D9-EF04-45CE-96F6-CE31022F4A2D}"/>
+  <xr:revisionPtr revIDLastSave="3696" documentId="13_ncr:1_{27CD5DFD-1054-4A33-AFFE-F35EA43968A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A72AD55D-9B9E-4104-87C1-9C41D55F1860}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="changelog input" sheetId="2" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2538" uniqueCount="1422">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2542" uniqueCount="1425">
   <si>
     <t>:base_ramp_storage_reserve
 :base_ramp_storage_envelopes
@@ -5250,30 +5250,42 @@
 configuration_envelopes_e_reserve_mu_v2</t>
   </si>
   <si>
+    <t>32.3s</t>
+  </si>
+  <si>
+    <t>4d26af57c</t>
+  </si>
+  <si>
+    <t>envelope
+configuration_envelopes_e_reserve_mu_v3</t>
+  </si>
+  <si>
+    <t>repo</t>
+  </si>
+  <si>
+    <t>RTS-GMLC_v2.1.3</t>
+  </si>
+  <si>
+    <t>net_demand = load</t>
+  </si>
+  <si>
     <t>from 2.4.1
 Renamed CSP and hydro reservoir asset resources
-configuration_envelopes_e_reserve_mu =  multiplier calculated based on Ax=B with B = max_{i&lt;=t} ER_{i,t}
+configuration_envelopes_e_reserve_mu =  multiplier calculated based on Ax=B with B = max_{i&lt;=t} ER_{i,t
 configuration_envelopes_e_reserve_mu_v2 =  multiplier calculated based on Ax=B with B = ER_{1,t}
-configuration_envelopes_e_reserve_mu_v3 =  multiplier calculated based on Ax=B with B = ER_{1,t} and clip[0,1]</t>
-  </si>
-  <si>
-    <t>32.3s</t>
-  </si>
-  <si>
-    <t>4d26af57c</t>
+configuration_envelopes_e_reserve_mu_v3 =  multiplier calculated based on Ax=B with B = ER_{1,t} and clip[0,1] --&gt; e_reserve_mu.py
+configuration_envelopes_cumulative_reserve_mu_v1.csv =  multiplier based on cumulative imbalance over reserves metodology -&gt; cumulative_reserve_mu.py. Multiplier as a function of time
+configuration_envelopes_cumulative_reserve_mu_v2.csv =  multiplier based on cumulative imbalance over reserves metodology -&gt; cumulative_reserve_mu.py. Multiplier as last hour's value from previous</t>
+  </si>
+  <si>
+    <t>32.4s</t>
+  </si>
+  <si>
+    <t>ab414</t>
   </si>
   <si>
     <t>envelope
-configuration_envelopes_e_reserve_mu_v3</t>
-  </si>
-  <si>
-    <t>repo</t>
-  </si>
-  <si>
-    <t>RTS-GMLC_v2.1.3</t>
-  </si>
-  <si>
-    <t>net_demand = load</t>
+configuration_envelopes_cumulative_reserve_mu_v2</t>
   </si>
 </sst>
 </file>
@@ -5553,10 +5565,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6200,10 +6208,10 @@
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
+        <v>1419</v>
+      </c>
+      <c r="C47" s="11" t="s">
         <v>1420</v>
-      </c>
-      <c r="C47" s="11" t="s">
-        <v>1421</v>
       </c>
     </row>
     <row r="48" spans="2:3" ht="90" x14ac:dyDescent="0.25">
@@ -6246,15 +6254,15 @@
         <v>1342</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" ht="150" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>1419</v>
+        <v>1418</v>
       </c>
       <c r="B53" s="43" t="s">
         <v>1361</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>1415</v>
+        <v>1421</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -6267,7 +6275,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>1419</v>
+        <v>1418</v>
       </c>
       <c r="B55" s="43" t="s">
         <v>1257</v>
@@ -15808,24 +15816,32 @@
     </row>
     <row r="580" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A580" s="15" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
       <c r="B580" s="13" t="s">
         <v>1361</v>
       </c>
       <c r="C580" s="13" t="s">
+        <v>1416</v>
+      </c>
+      <c r="D580" s="25" t="s">
         <v>1417</v>
       </c>
-      <c r="D580" s="25" t="s">
-        <v>1418</v>
-      </c>
       <c r="E580" s="13"/>
     </row>
-    <row r="581" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A581" s="13"/>
-      <c r="B581" s="13"/>
-      <c r="C581" s="13"/>
-      <c r="D581" s="14"/>
+    <row r="581" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A581" s="13" t="s">
+        <v>1422</v>
+      </c>
+      <c r="B581" s="13" t="s">
+        <v>1361</v>
+      </c>
+      <c r="C581" s="13" t="s">
+        <v>1423</v>
+      </c>
+      <c r="D581" s="25" t="s">
+        <v>1424</v>
+      </c>
       <c r="E581" s="13"/>
     </row>
     <row r="582" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>